<commit_message>
12 June - with code guide
Working code - After 100% utilization of GitHub
</commit_message>
<xml_diff>
--- a/Ref docs/Resource/Deloyment_pool_update.xlsx
+++ b/Ref docs/Resource/Deloyment_pool_update.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rockwellautomation-my.sharepoint.com/personal/anjana_sharma_rockwellautomation_com/Documents/Anjana Sharma - All Important Documents/1. My work/RA Work/AM-APP/Ref docs/Resource/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{C42A48F7-6787-4F13-A89B-C131E85EF6B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{942A20D9-53B4-45F4-88A3-EE3ED6A391F4}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{C42A48F7-6787-4F13-A89B-C131E85EF6B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2B2EDA5-AF2F-48D0-AD43-467B193A9CB5}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -456,7 +456,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:C97"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
@@ -531,7 +530,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" hidden="1">
+    <row r="7" spans="1:3">
       <c r="A7" s="1">
         <v>90719559</v>
       </c>
@@ -542,7 +541,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:3" hidden="1">
+    <row r="8" spans="1:3">
       <c r="A8" s="1">
         <v>90719892</v>
       </c>
@@ -619,7 +618,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1">
+    <row r="15" spans="1:3">
       <c r="A15" s="1">
         <v>90719885</v>
       </c>
@@ -652,7 +651,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" hidden="1">
+    <row r="18" spans="1:3">
       <c r="A18" s="1">
         <v>20072996</v>
       </c>
@@ -696,7 +695,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:3" hidden="1">
+    <row r="22" spans="1:3">
       <c r="A22" s="1">
         <v>90732309</v>
       </c>
@@ -718,7 +717,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:3" hidden="1">
+    <row r="24" spans="1:3">
       <c r="A24" s="1">
         <v>90725487</v>
       </c>
@@ -740,7 +739,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:3" hidden="1">
+    <row r="26" spans="1:3">
       <c r="A26" s="1">
         <v>90719413</v>
       </c>
@@ -751,7 +750,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:3" hidden="1">
+    <row r="27" spans="1:3">
       <c r="A27" s="1">
         <v>90719527</v>
       </c>
@@ -762,7 +761,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:3" hidden="1">
+    <row r="28" spans="1:3">
       <c r="A28" s="1">
         <v>90719879</v>
       </c>
@@ -773,7 +772,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" hidden="1">
+    <row r="29" spans="1:3">
       <c r="A29" s="1">
         <v>90732691</v>
       </c>
@@ -806,7 +805,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:3" hidden="1">
+    <row r="32" spans="1:3">
       <c r="A32" s="1">
         <v>90719900</v>
       </c>
@@ -817,7 +816,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:3" hidden="1">
+    <row r="33" spans="1:3">
       <c r="A33" s="1">
         <v>90719932</v>
       </c>
@@ -861,7 +860,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:3" hidden="1">
+    <row r="37" spans="1:3">
       <c r="A37" s="1">
         <v>90719710</v>
       </c>
@@ -894,7 +893,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:3" hidden="1">
+    <row r="40" spans="1:3">
       <c r="A40" s="1">
         <v>90727248</v>
       </c>
@@ -916,7 +915,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:3" hidden="1">
+    <row r="42" spans="1:3">
       <c r="A42" s="1">
         <v>90727178</v>
       </c>
@@ -927,7 +926,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:3" hidden="1">
+    <row r="43" spans="1:3">
       <c r="A43" s="1">
         <v>90727247</v>
       </c>
@@ -938,7 +937,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:3" hidden="1">
+    <row r="44" spans="1:3">
       <c r="A44" s="1">
         <v>90719916</v>
       </c>
@@ -1004,7 +1003,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="50" spans="1:3" hidden="1">
+    <row r="50" spans="1:3">
       <c r="A50" s="1">
         <v>90727544</v>
       </c>
@@ -1015,7 +1014,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:3" hidden="1">
+    <row r="51" spans="1:3">
       <c r="A51" s="1">
         <v>90719735</v>
       </c>
@@ -1037,7 +1036,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:3" hidden="1">
+    <row r="53" spans="1:3">
       <c r="A53" s="1">
         <v>90719862</v>
       </c>
@@ -1048,7 +1047,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="54" spans="1:3" hidden="1">
+    <row r="54" spans="1:3">
       <c r="A54" s="1">
         <v>90727174</v>
       </c>
@@ -1070,7 +1069,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="56" spans="1:3" hidden="1">
+    <row r="56" spans="1:3">
       <c r="A56" s="1">
         <v>90718853</v>
       </c>
@@ -1092,7 +1091,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:3" hidden="1">
+    <row r="58" spans="1:3">
       <c r="A58" s="1">
         <v>90719008</v>
       </c>
@@ -1136,7 +1135,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="62" spans="1:3" hidden="1">
+    <row r="62" spans="1:3">
       <c r="A62" s="1">
         <v>90732280</v>
       </c>
@@ -1147,7 +1146,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="1:3" hidden="1">
+    <row r="63" spans="1:3">
       <c r="A63" s="1">
         <v>90725456</v>
       </c>
@@ -1158,7 +1157,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="1:3" hidden="1">
+    <row r="64" spans="1:3">
       <c r="A64" s="1">
         <v>90732412</v>
       </c>
@@ -1235,7 +1234,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:3" hidden="1">
+    <row r="71" spans="1:3">
       <c r="A71" s="1">
         <v>90719316</v>
       </c>
@@ -1257,7 +1256,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:3" hidden="1">
+    <row r="73" spans="1:3">
       <c r="A73" s="1">
         <v>90719569</v>
       </c>
@@ -1279,7 +1278,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="75" spans="1:3" hidden="1">
+    <row r="75" spans="1:3">
       <c r="A75" s="1">
         <v>90732448</v>
       </c>
@@ -1312,7 +1311,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:3" hidden="1">
+    <row r="78" spans="1:3">
       <c r="A78" s="1">
         <v>90719796</v>
       </c>
@@ -1323,7 +1322,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:3" hidden="1">
+    <row r="79" spans="1:3">
       <c r="A79" s="1">
         <v>90719452</v>
       </c>
@@ -1378,7 +1377,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="84" spans="1:3" hidden="1">
+    <row r="84" spans="1:3">
       <c r="A84" s="1">
         <v>90719880</v>
       </c>
@@ -1411,7 +1410,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="87" spans="1:3" hidden="1">
+    <row r="87" spans="1:3">
       <c r="A87" s="1">
         <v>90732269</v>
       </c>
@@ -1433,7 +1432,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="89" spans="1:3" hidden="1">
+    <row r="89" spans="1:3">
       <c r="A89" s="1">
         <v>90719396</v>
       </c>
@@ -1477,7 +1476,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="93" spans="1:3" hidden="1">
+    <row r="93" spans="1:3">
       <c r="A93" s="1">
         <v>90719522</v>
       </c>
@@ -1499,7 +1498,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="95" spans="1:3" hidden="1">
+    <row r="95" spans="1:3">
       <c r="A95" s="1">
         <v>90732271</v>
       </c>
@@ -1521,7 +1520,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="97" spans="1:3" hidden="1">
+    <row r="97" spans="1:3">
       <c r="A97" s="1">
         <v>90724646</v>
       </c>
@@ -1533,14 +1532,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C97" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Notice"/>
-        <filter val="Proposed"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:C97" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>